<commit_message>
quality report of missing variables in 2015 data set checking about at least one variable was missing
</commit_message>
<xml_diff>
--- a/notebooks/2015_Birth/First stage 2015/01_missing_values.xlsx
+++ b/notebooks/2015_Birth/First stage 2015/01_missing_values.xlsx
@@ -504,68 +504,68 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Multiple_Birth_Status</t>
+          <t>Birth_Weight(grams)</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>332393</v>
+        <v>33604</v>
       </c>
       <c r="C2" s="3" t="n">
-        <v>98.90000000000001</v>
+        <v>10</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="E2" s="3" t="n">
-        <v>3</v>
+        <v>1760</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>3704</v>
+        <v>302493</v>
       </c>
       <c r="G2" s="3" t="n">
-        <v>1.1</v>
+        <v>90</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Birth_Weight(grams)</t>
+          <t>Race_of_Father</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>33604</v>
+        <v>221</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>10</v>
+        <v>0.1</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="E3" s="3" t="n">
-        <v>1760</v>
+        <v>12</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>302493</v>
+        <v>335876</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>90</v>
+        <v>99.90000000000001</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Race_of_Father</t>
+          <t>Birth_Order</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>221</v>
+        <v>1</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -573,37 +573,37 @@
         </is>
       </c>
       <c r="E4" s="3" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>335876</v>
+        <v>336096</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>99.90000000000001</v>
+        <v>100</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Birth_Order</t>
+          <t>Registered_Year</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>int64</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="E5" s="3" t="n">
-        <v>9</v>
-      </c>
       <c r="F5" s="3" t="n">
-        <v>336096</v>
+        <v>336097</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>100</v>
@@ -639,7 +639,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Registered_Year</t>
+          <t>Registered_Year 2.0</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
@@ -666,7 +666,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Registered_Year 2.0</t>
+          <t>Birth_Year_2.0</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
@@ -681,7 +681,7 @@
         </is>
       </c>
       <c r="E8" s="3" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="F8" s="3" t="n">
         <v>336097</v>
@@ -855,7 +855,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Birth_Year_2.0</t>
+          <t>Multiple_Birth_Status</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
@@ -866,11 +866,11 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
-        <v>60</v>
+        <v>4</v>
       </c>
       <c r="F15" s="3" t="n">
         <v>336097</v>
@@ -1044,7 +1044,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5">
@@ -1054,7 +1054,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>366219</v>
+        <v>33826</v>
       </c>
     </row>
     <row r="6">
@@ -1064,7 +1064,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>6.05</v>
+        <v>0.5600000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
creating complete data files 2015
</commit_message>
<xml_diff>
--- a/notebooks/2015_Birth/First stage 2015/01_missing_values.xlsx
+++ b/notebooks/2015_Birth/First stage 2015/01_missing_values.xlsx
@@ -452,7 +452,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>33604</v>
+        <v>33639</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>10</v>
@@ -522,7 +522,7 @@
         <v>1760</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>302493</v>
+        <v>302458</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>90</v>
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>221</v>
+        <v>280</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>0.1</v>
@@ -549,7 +549,7 @@
         <v>12</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>335876</v>
+        <v>335817</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>99.90000000000001</v>
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>1</v>
+        <v>60</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>0</v>
@@ -576,7 +576,7 @@
         <v>9</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>336096</v>
+        <v>336037</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>100</v>
@@ -589,21 +589,21 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="E5" s="3" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>336097</v>
+        <v>336038</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>100</v>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>0</v>
@@ -630,7 +630,7 @@
         <v>12</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>336097</v>
+        <v>336038</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>100</v>
@@ -639,25 +639,25 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Registered_Year 2.0</t>
+          <t>Birth_Month</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>336097</v>
+        <v>336038</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>100</v>
@@ -666,25 +666,25 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Birth_Year_2.0</t>
+          <t>Registered_District</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>336097</v>
+        <v>336038</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>100</v>
@@ -693,25 +693,25 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Registered_District</t>
+          <t>Birh_Year</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="C9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
-        <v>25</v>
+        <v>60</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>336097</v>
+        <v>336038</v>
       </c>
       <c r="G9" s="3" t="n">
         <v>100</v>
@@ -720,25 +720,25 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Birh_Year</t>
+          <t>Birh_Year 2.0</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="C10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
         <v>60</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>336097</v>
+        <v>336038</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>100</v>
@@ -747,25 +747,25 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Birth_Month</t>
+          <t>Twin</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="C11" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>336097</v>
+        <v>336038</v>
       </c>
       <c r="G11" s="3" t="n">
         <v>100</v>
@@ -774,25 +774,25 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>TWIN</t>
+          <t>Hospital or Not</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="C12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>336097</v>
+        <v>336038</v>
       </c>
       <c r="G12" s="3" t="n">
         <v>100</v>
@@ -801,11 +801,11 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Hospital or Not</t>
+          <t xml:space="preserve">Gender </t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="C13" s="3" t="n">
         <v>0</v>
@@ -819,7 +819,7 @@
         <v>2</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>336097</v>
+        <v>336038</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>100</v>
@@ -828,11 +828,11 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Gender</t>
+          <t>Multiple_Birth_Status</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="C14" s="3" t="n">
         <v>0</v>
@@ -843,10 +843,10 @@
         </is>
       </c>
       <c r="E14" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>336097</v>
+        <v>336038</v>
       </c>
       <c r="G14" s="3" t="n">
         <v>100</v>
@@ -855,25 +855,25 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Multiple_Birth_Status</t>
+          <t>Age of Mother</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="C15" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>float64</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
-        <v>4</v>
+        <v>41</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>336097</v>
+        <v>336038</v>
       </c>
       <c r="G15" s="3" t="n">
         <v>100</v>
@@ -882,25 +882,25 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Age of Mother</t>
+          <t>Marital_Status</t>
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="C16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
-        <v>41</v>
+        <v>2</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>336097</v>
+        <v>336038</v>
       </c>
       <c r="G16" s="3" t="n">
         <v>100</v>
@@ -909,11 +909,11 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Marital_Status</t>
+          <t>District_of_Mother</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="C17" s="3" t="n">
         <v>0</v>
@@ -924,10 +924,10 @@
         </is>
       </c>
       <c r="E17" s="3" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>336097</v>
+        <v>336038</v>
       </c>
       <c r="G17" s="3" t="n">
         <v>100</v>
@@ -936,11 +936,11 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>District_of_Mother</t>
+          <t>Race_of_Mother</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
-        <v>0</v>
+        <v>59</v>
       </c>
       <c r="C18" s="3" t="n">
         <v>0</v>
@@ -951,39 +951,12 @@
         </is>
       </c>
       <c r="E18" s="3" t="n">
-        <v>26</v>
+        <v>12</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>336097</v>
+        <v>336038</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Race_of_Mother</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="C19" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>str</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="F19" s="3" t="n">
-        <v>336097</v>
-      </c>
-      <c r="G19" s="3" t="n">
         <v>100</v>
       </c>
     </row>
@@ -1034,7 +1007,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4">
@@ -1044,7 +1017,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>3</v>
+        <v>17</v>
       </c>
     </row>
     <row r="5">
@@ -1054,7 +1027,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>33826</v>
+        <v>34805</v>
       </c>
     </row>
     <row r="6">
@@ -1064,7 +1037,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.61</v>
       </c>
     </row>
   </sheetData>

</xml_diff>